<commit_message>
Dummy push converter for static bicycle parking data
</commit_message>
<xml_diff>
--- a/tests/converters/data/dummy_bike.xlsx
+++ b/tests/converters/data/dummy_bike.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FTL\FTLBank\ipl\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243F4444-A413-4633-A9D5-D2E0D25FC92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F468CBC7-DA21-47CE-8D1E-D7F04DCFD7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{80802002-80FC-40E1-8B8F-C25AD4FD32B4}"/>
   </bookViews>
@@ -246,7 +246,7 @@
   <numFmts count="1">
     <numFmt numFmtId="169" formatCode="&quot;Wahr&quot;;&quot;Falsch&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,6 +284,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -314,7 +322,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -329,10 +337,11 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -720,7 +729,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:36" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
@@ -747,7 +756,7 @@
       <c r="I1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="9" t="s">
         <v>60</v>
       </c>
       <c r="K1" s="7" t="s">
@@ -762,28 +771,28 @@
       <c r="N1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="9" t="s">
         <v>62</v>
       </c>
       <c r="P1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="8" t="s">
         <v>55</v>
       </c>
       <c r="S1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="T1" s="9" t="s">
         <v>15</v>
       </c>
       <c r="U1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="V1" s="9" t="s">
         <v>17</v>
       </c>
       <c r="W1" s="7" t="s">
@@ -816,16 +825,16 @@
       <c r="AF1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="AG1" s="7" t="s">
+      <c r="AG1" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="AH1" s="7" t="s">
+      <c r="AH1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="AI1" s="8" t="s">
+      <c r="AI1" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="AJ1" s="7" t="s">
+      <c r="AJ1" s="9" t="s">
         <v>65</v>
       </c>
     </row>

</xml_diff>